<commit_message>
fix(dlaa): drop false Honda Fit from English "Fit For" titles
</commit_message>
<xml_diff>
--- a/catalogos/dlaa/catalogo.xlsx
+++ b/catalogos/dlaa/catalogo.xlsx
@@ -2704,7 +2704,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>NISSAN, TOYOTA | Frontier, X-Trail, Roomy, Rogue, FIT | 2021-ON</t>
+          <t>NISSAN, TOYOTA | Frontier, X-Trail, Roomy, Rogue | 2021-ON</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>TOYOTA | 4Runner, Probox, Prious, Baqua, FIT | 2018-2019</t>
+          <t>TOYOTA | 4Runner, Probox, Prious, Baqua | 2018-2019</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>TOYOTA | C-Hr, FIT | 2017-2019</t>
+          <t>TOYOTA | C-Hr | 2017-2019</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">

</xml_diff>